<commit_message>
feat: expand battle systems and testing tools
</commit_message>
<xml_diff>
--- a/DataTables/Datas/#BuffInfo.xlsx
+++ b/DataTables/Datas/#BuffInfo.xlsx
@@ -422,7 +422,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I29"/>
+  <dimension ref="A1:I30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1429,6 +1429,42 @@
         <v>0</v>
       </c>
     </row>
+    <row r="30">
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Morale</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>士气</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>特殊增益，当前 {V} 层</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>UI/Buff/Icon_Morale</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>Buff</t>
+        </is>
+      </c>
+      <c r="G30" t="n">
+        <v>-1</v>
+      </c>
+      <c r="H30" t="n">
+        <v>3</v>
+      </c>
+      <c r="I30" t="b">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>